<commit_message>
Génère le PDF du MOADR (bandeaux navy, tableau réel section 5.2)
Même langage visuel que le RePSS (bandeaux de titre bleu marine, sections
encadrées) sur une feuille de styles autonome (pas de partage avec
RepssDocument.jsx, pour ne pas toucher au PDF RePSS déjà en production sur
un document structurellement différent). Tableau paysage pour la section
5.2 (Réf./Tâche/Danger/Situation dangereuse/Mesures/P/E/G/Score/Niveau),
couleur de la cellule dérivée du même niveauDepuisScore que le formulaire.

Référence MOADR-{année}-{XXXXX} attribuée seulement au moment de la
génération (bouton en deux temps : "Générer le PDF" attribue la référence
puis affiche le vrai lien de téléchargement), même principe que
meta.repssNumero.

Reste à faire : intégration avec les demandesMoadr d'un RePSS
(pré-remplissage + jointure du PDF généré en annexe).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFXiTptZrjH4tqXxgg3KiT
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G463"/>
+  <dimension ref="A1:G464"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -16123,6 +16123,38 @@
         </is>
       </c>
     </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>moadr_voir_tableau_page_suivante</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Voir le tableau détaillé, page suivante.</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>See the detailed table on the next page.</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Zie de gedetailleerde tabel op de volgende pagina.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ajoute l'import de fichier au MOADR, détaille l'explication Kinney (P/E/G)
"Importer un fichier" en haut de l'écran MOADR (même mécanisme que
"Reprendre un RePSS existant", §8) : jusqu'ici le bouton "Enregistrer"
existait sans aucun moyen de recharger le .json produit.

Remplace la mention "sur la même échelle que le reste des documents RePSS
(voir Annexe 1 — Légende Kinney)" par la définition des trois facteurs
(Probabilité, Exposition, Gravité) dans l'encadré d'introduction, web et
PDF, à la demande de Ced.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFXiTptZrjH4tqXxgg3KiT
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G466"/>
+  <dimension ref="A1:G475"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -15021,17 +15021,17 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>La méthode Kinney quantifie chaque risque à partir de trois facteurs : Probabilité, Exposition et Gravité. Le risque est calculé selon la formule R = Probabilité × Exposition × Gravité, sur la même échelle que le reste des documents RePSS (voir Annexe 1 — Légende Kinney).</t>
+          <t>La méthode Kinney quantifie chaque risque à partir de trois facteurs : Probabilité, Exposition et Gravité. Le risque est calculé selon la formule R = Probabilité × Exposition × Gravité.</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>The Kinney method quantifies each risk from three factors: Probability, Exposure and Severity. The risk is calculated using the formula R = Probability × Exposure × Severity, on the same scale as the rest of the RePSS documents (see Appendix 1 — Kinney Legend).</t>
+          <t>The Kinney method quantifies each risk from three factors: Probability, Exposure and Severity. The risk is calculated using the formula R = Probability × Exposure × Severity.</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t>De Kinney-methode kwantificeert elk risico aan de hand van drie factoren: Waarschijnlijkheid, Blootstelling en Ernst. Het risico wordt berekend met de formule R = Waarschijnlijkheid × Blootstelling × Ernst, op dezelfde schaal als de rest van de RePSS-documenten (zie Bijlage 1 — Kinney-legende).</t>
+          <t>De Kinney-methode kwantificeert elk risico aan de hand van drie factoren: Waarschijnlijkheid, Blootstelling en Ernst. Het risico wordt berekend met de formule R = Waarschijnlijkheid × Blootstelling × Ernst.</t>
         </is>
       </c>
     </row>
@@ -16216,6 +16216,294 @@
       <c r="F466" t="inlineStr">
         <is>
           <t>MOADR heropenen</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>moadr_kinney_p_titre</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Facteur de probabilité (P)</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Probability factor (P)</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Waarschijnlijkheidsfactor (P)</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>moadr_kinney_p_texte</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>La probabilité est le risque qu'un danger entraîne des dommages. Vous devez procéder à cette estimation sans tenir compte des mesures de prévention individuelles ou collectives.</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Probability is the risk that a hazard results in harm. This estimate must be made without taking individual or collective prevention measures into account.</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Waarschijnlijkheid is het risico dat een gevaar tot schade leidt. Deze inschatting moet gebeuren zonder rekening te houden met individuele of collectieve preventiemaatregelen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>moadr_kinney_e_titre</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Facteur d'exposition (E)</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Exposure factor (E)</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Blootstellingsfactor (E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>moadr_kinney_e_texte</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Le facteur d'exposition tient compte de la durée et de la fréquence de l'exposition au danger.</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>The exposure factor takes into account the duration and frequency of exposure to the hazard.</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>De blootstellingsfactor houdt rekening met de duur en de frequentie van de blootstelling aan het gevaar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>moadr_kinney_g_titre</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Degré de gravité (G)</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Severity level (G)</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Ernstgraad (G)</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>moadr_kinney_g_texte</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Pour estimer le degré de gravité, vous devez estimer les plus graves effets éventuels de l'exposition.</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>To estimate the severity level, you must estimate the most serious possible effects of the exposure.</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Om de ernstgraad in te schatten, moet u de ernstigste mogelijke gevolgen van de blootstelling inschatten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>moadr_importer_bouton</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Importer un fichier</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Import a file</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Een bestand importeren</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>moadr_importer_erreur</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Fichier invalide : ce n'est pas un MOADR (.json).</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Invalid file: this is not a MOADR (.json).</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Ongeldig bestand: dit is geen MOADR (.json).</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>moadr_importer_succes</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>MOADR</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>MOADR importé.</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>MOADR imported.</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>MOADR geïmporteerd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige le signe du critère "heures de chantier" en Caractérisation
"Heures de chantier < 1000" → "> 1000" : le signe était inversé, cohérent
avec l'avertissement du document de référence de l'abrégé ("interdiction
d'utiliser l'abrégé pour les chantiers dont le total des heures prestées
par vma sud serait supérieur à 1000 heures"). Renomme aussi le champ
interne heuresInf1000 → heuresSup1000 (dossier.js, Caracterisation.jsx,
CLAUDE.md §3/§5) pour que le nom reflète ce qu'il signifie réellement.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFXiTptZrjH4tqXxgg3KiT
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -8044,17 +8044,17 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Heures de chantier &lt; 1000</t>
+          <t>Heures de chantier &gt; 1000</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Site hours &lt; 1000</t>
+          <t>Site hours &gt; 1000</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Werfuren &lt; 1000</t>
+          <t>Werfuren &gt; 1000</t>
         </is>
       </c>
     </row>

</xml_diff>